<commit_message>
cambios en table mod
</commit_message>
<xml_diff>
--- a/tests/output_frame.xlsx
+++ b/tests/output_frame.xlsx
@@ -16,10 +16,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
   <si>
-    <t>region</t>
+    <t>venta</t>
   </si>
   <si>
-    <t>venta</t>
+    <t>region</t>
   </si>
   <si>
     <t>norte</t>
@@ -387,51 +387,51 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" t="s">
+      <c r="A2">
+        <v>100</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
-        <v>100</v>
-      </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" t="s">
+      <c r="A3">
+        <v>200</v>
+      </c>
+      <c r="B3" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
-        <v>200</v>
-      </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" t="s">
+      <c r="A4">
+        <v>300</v>
+      </c>
+      <c r="B4" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
-        <v>300</v>
-      </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" t="s">
+      <c r="A5">
+        <v>400</v>
+      </c>
+      <c r="B5" t="s">
         <v>3</v>
       </c>
-      <c r="B5">
-        <v>400</v>
-      </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" t="s">
+      <c r="A6">
+        <v>500</v>
+      </c>
+      <c r="B6" t="s">
         <v>4</v>
       </c>
-      <c r="B6">
-        <v>500</v>
-      </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" t="s">
+      <c r="A7">
+        <v>600</v>
+      </c>
+      <c r="B7" t="s">
         <v>4</v>
-      </c>
-      <c r="B7">
-        <v>600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cambios en table mod table
</commit_message>
<xml_diff>
--- a/tests/output_frame.xlsx
+++ b/tests/output_frame.xlsx
@@ -16,10 +16,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="5">
   <si>
-    <t>venta</t>
+    <t>region</t>
   </si>
   <si>
-    <t>region</t>
+    <t>venta</t>
   </si>
   <si>
     <t>norte</t>
@@ -387,51 +387,51 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
         <v>100</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3">
+      <c r="B3">
         <v>200</v>
       </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4">
         <v>300</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5">
+      <c r="B5">
         <v>400</v>
       </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
         <v>500</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7">
+      <c r="B7">
         <v>600</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>